<commit_message>
DBからの設定項目(required , transform = trim)に対応
</commit_message>
<xml_diff>
--- a/internal/excel/Book1.xlsx
+++ b/internal/excel/Book1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\right\dev\excel-template-mapper\internal\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EBA5A17-12EA-4EAC-A276-80691579F039}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADDAB97B-B045-4421-9CA7-869AA8C5DF50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17520" yWindow="7695" windowWidth="43200" windowHeight="23445" xr2:uid="{FDF70F5C-09E2-44A8-BC50-9E466331B047}"/>
+    <workbookView xWindow="57480" yWindow="13395" windowWidth="29040" windowHeight="15720" xr2:uid="{FDF70F5C-09E2-44A8-BC50-9E466331B047}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,15 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
-  <si>
-    <t>いいい</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>ううう</t>
-    <phoneticPr fontId="1"/>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>dddd</t>
     <phoneticPr fontId="1"/>
@@ -81,23 +73,23 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>あああ</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>えええ</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>aaajj</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>bbb</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
     <t>cccc</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>aaaa</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> あああ</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -144,8 +136,11 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -484,47 +479,47 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFA2F540-7B08-4537-AF23-4359F7637B02}">
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="3" max="3" width="13.5" style="1" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>4</v>
-      </c>
-      <c r="C1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" t="s">
-        <v>1</v>
+        <v>9</v>
+      </c>
+      <c r="C2" s="1">
+        <v>46061.628472222219</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>11</v>
+        <v>6</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>